<commit_message>
Added data validation for Excel input data
</commit_message>
<xml_diff>
--- a/workspaces/example_new_calculations/input/input.xlsx
+++ b/workspaces/example_new_calculations/input/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MKL\Documents\Github\GeoProb-Pipe\workspaces\example_new_calculations\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB9AABB1-8C0C-43A9-B9D2-267F6B69BDF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0624654-91F0-4134-87DE-988E2AA5D3E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-180" windowWidth="29040" windowHeight="17520" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
+    <workbookView xWindow="38280" yWindow="-165" windowWidth="25440" windowHeight="15270" activeTab="2" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
   </bookViews>
   <sheets>
     <sheet name="Vakken" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,9 @@
     <sheet name="Ondergrondscenarios" sheetId="3" r:id="rId3"/>
     <sheet name="Overzicht_variabelen" sheetId="2" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Ondergrondscenarios!$A$1:$O$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="750" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="209">
   <si>
     <t>M_van</t>
   </si>
@@ -687,7 +690,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -697,6 +700,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -713,13 +722,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -827,7 +838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{ECE0F829-0060-4D7E-94D4-430EA87FED82}" name="Tabel12" displayName="Tabel12" ref="A2:P55" headerRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{ECE0F829-0060-4D7E-94D4-430EA87FED82}" name="Tabel12" displayName="Tabel12" ref="A2:P69" headerRowCount="0" totalsRowShown="0">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P55">
     <sortCondition ref="D2:D55" customList="Input,Input,can also be calculated,Constant,Calculated"/>
     <sortCondition ref="A2:A55"/>
@@ -1172,21 +1183,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93C253AA-AAA1-47E5-9332-CA169F978D7A}">
   <dimension ref="A1:K10"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.25" customWidth="1"/>
-    <col min="2" max="2" width="32.875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="8.25" customWidth="1"/>
-    <col min="5" max="5" width="8.75" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.375" customWidth="1"/>
+    <col min="1" max="1" width="8.19921875" customWidth="1"/>
+    <col min="2" max="2" width="32.8984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="8.19921875" customWidth="1"/>
+    <col min="5" max="5" width="8.69921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.8984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.09765625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.3984375" customWidth="1"/>
     <col min="10" max="10" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.75" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>180</v>
       </c>
@@ -1211,19 +1222,19 @@
       <c r="H1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="4" t="str">
-        <f>LEFT(H1,LEN(H1)-5)&amp;VLOOKUP(LEFT(H1,LEN(H1)-5),Overzicht_variabelen!$A$2:$F$55,6,(FALSE))</f>
+      <c r="I1" s="6" t="str">
+        <f>LEFT(H1,LEN(H1)-5)&amp;VLOOKUP(LEFT(H1,LEN(H1)-5),Overzicht_variabelen!$A$2:$F$69,6,(FALSE))</f>
         <v>c_voorland_stdev</v>
       </c>
       <c r="J1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="4" t="str">
-        <f>LEFT(J1,LEN(J1)-5)&amp;VLOOKUP(LEFT(J1,LEN(J1)-5),Overzicht_variabelen!$A$2:$F$55,6,(FALSE))</f>
+      <c r="K1" s="6" t="str">
+        <f>LEFT(J1,LEN(J1)-5)&amp;VLOOKUP(LEFT(J1,LEN(J1)-5),Overzicht_variabelen!$A$2:$F$69,6,(FALSE))</f>
         <v>c_achterland_vc</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1258,7 +1269,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1293,7 +1304,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1328,7 +1339,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1363,7 +1374,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1398,7 +1409,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1433,7 +1444,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1468,7 +1479,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1503,7 +1514,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1549,25 +1560,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AB77777-746E-45C0-BE11-D138C11C003A}">
   <dimension ref="A1:T103"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.375" customWidth="1"/>
+    <col min="1" max="1" width="7.3984375" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="19.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="19.3984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.8984375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.25" customWidth="1"/>
-    <col min="11" max="11" width="19.25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.625" bestFit="1" customWidth="1"/>
-    <col min="15" max="20" width="17.75" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.3984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.8984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.19921875" customWidth="1"/>
+    <col min="11" max="11" width="19.19921875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.09765625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.8984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.59765625" bestFit="1" customWidth="1"/>
+    <col min="15" max="20" width="17.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>180</v>
       </c>
@@ -1613,26 +1624,26 @@
       <c r="O1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="P1" s="4" t="str">
-        <f>LEFT(O1,LEN(O1)-5)&amp;VLOOKUP(LEFT(O1,LEN(O1)-5),Overzicht_variabelen!$A$2:$F$55,6,(FALSE))</f>
+      <c r="P1" s="6" t="str">
+        <f>LEFT(O1,LEN(O1)-5)&amp;VLOOKUP(LEFT(O1,LEN(O1)-5),Overzicht_variabelen!$A$2:$F$69,6,(FALSE))</f>
         <v>modelfactor_u_stdev</v>
       </c>
       <c r="Q1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="R1" s="4" t="str">
-        <f>LEFT(Q1,LEN(Q1)-5)&amp;VLOOKUP(LEFT(Q1,LEN(Q1)-5),Overzicht_variabelen!$A$2:$F$55,6,(FALSE))</f>
+      <c r="R1" s="6" t="str">
+        <f>LEFT(Q1,LEN(Q1)-5)&amp;VLOOKUP(LEFT(Q1,LEN(Q1)-5),Overzicht_variabelen!$A$2:$F$69,6,(FALSE))</f>
         <v>modelfactor_h_stdev</v>
       </c>
       <c r="S1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="T1" s="4" t="str">
-        <f>LEFT(S1,LEN(S1)-5)&amp;VLOOKUP(LEFT(S1,LEN(S1)-5),Overzicht_variabelen!$A$2:$F$55,6,(FALSE))</f>
+      <c r="T1" s="6" t="str">
+        <f>LEFT(S1,LEN(S1)-5)&amp;VLOOKUP(LEFT(S1,LEN(S1)-5),Overzicht_variabelen!$A$2:$F$69,6,(FALSE))</f>
         <v>modelfactor_p_stdev</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1694,7 +1705,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>3</v>
       </c>
@@ -1756,7 +1767,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>4</v>
       </c>
@@ -1818,7 +1829,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1880,7 +1891,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
@@ -1942,7 +1953,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2004,7 +2015,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>5</v>
       </c>
@@ -2066,7 +2077,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>5</v>
       </c>
@@ -2128,7 +2139,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>5</v>
       </c>
@@ -2190,7 +2201,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>5</v>
       </c>
@@ -2252,7 +2263,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>5</v>
       </c>
@@ -2314,7 +2325,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>5</v>
       </c>
@@ -2376,7 +2387,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>5</v>
       </c>
@@ -2438,7 +2449,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>5</v>
       </c>
@@ -2500,7 +2511,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>5</v>
       </c>
@@ -2562,7 +2573,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>6</v>
       </c>
@@ -2624,7 +2635,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>6</v>
       </c>
@@ -2686,7 +2697,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>6</v>
       </c>
@@ -2748,7 +2759,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>6</v>
       </c>
@@ -2810,7 +2821,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>6</v>
       </c>
@@ -2872,7 +2883,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>6</v>
       </c>
@@ -2934,7 +2945,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>6</v>
       </c>
@@ -2996,7 +3007,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>6</v>
       </c>
@@ -3058,7 +3069,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>6</v>
       </c>
@@ -3120,7 +3131,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>7</v>
       </c>
@@ -3182,7 +3193,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>7</v>
       </c>
@@ -3244,7 +3255,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>7</v>
       </c>
@@ -3306,7 +3317,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>7</v>
       </c>
@@ -3368,7 +3379,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>7</v>
       </c>
@@ -3430,7 +3441,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>7</v>
       </c>
@@ -3492,7 +3503,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>7</v>
       </c>
@@ -3554,7 +3565,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>7</v>
       </c>
@@ -3616,7 +3627,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>7</v>
       </c>
@@ -3678,7 +3689,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>7</v>
       </c>
@@ -3740,7 +3751,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>7</v>
       </c>
@@ -3802,7 +3813,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>7</v>
       </c>
@@ -3864,7 +3875,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>7</v>
       </c>
@@ -3926,7 +3937,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>7</v>
       </c>
@@ -3988,7 +3999,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>7</v>
       </c>
@@ -4050,7 +4061,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>8</v>
       </c>
@@ -4112,7 +4123,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>8</v>
       </c>
@@ -4174,7 +4185,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>8</v>
       </c>
@@ -4236,7 +4247,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>8</v>
       </c>
@@ -4298,7 +4309,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>8</v>
       </c>
@@ -4360,7 +4371,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>8</v>
       </c>
@@ -4422,7 +4433,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>8</v>
       </c>
@@ -4484,7 +4495,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>8</v>
       </c>
@@ -4546,7 +4557,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>8</v>
       </c>
@@ -4608,7 +4619,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>8</v>
       </c>
@@ -4670,7 +4681,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>8</v>
       </c>
@@ -4732,7 +4743,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>8</v>
       </c>
@@ -4794,7 +4805,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>8</v>
       </c>
@@ -4856,7 +4867,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>8</v>
       </c>
@@ -4918,7 +4929,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>8</v>
       </c>
@@ -4980,7 +4991,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>8</v>
       </c>
@@ -5042,7 +5053,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>8</v>
       </c>
@@ -5104,7 +5115,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>8</v>
       </c>
@@ -5166,7 +5177,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>8</v>
       </c>
@@ -5228,7 +5239,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>8</v>
       </c>
@@ -5290,7 +5301,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>8</v>
       </c>
@@ -5352,7 +5363,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>8</v>
       </c>
@@ -5414,7 +5425,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>8</v>
       </c>
@@ -5476,7 +5487,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>8</v>
       </c>
@@ -5538,7 +5549,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>8</v>
       </c>
@@ -5600,7 +5611,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>8</v>
       </c>
@@ -5662,7 +5673,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>8</v>
       </c>
@@ -5724,7 +5735,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>8</v>
       </c>
@@ -5786,7 +5797,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>8</v>
       </c>
@@ -5848,7 +5859,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>8</v>
       </c>
@@ -5910,7 +5921,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>8</v>
       </c>
@@ -5972,7 +5983,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>8</v>
       </c>
@@ -6034,7 +6045,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>8</v>
       </c>
@@ -6096,7 +6107,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>8</v>
       </c>
@@ -6158,7 +6169,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>8</v>
       </c>
@@ -6220,7 +6231,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>8</v>
       </c>
@@ -6282,7 +6293,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>8</v>
       </c>
@@ -6344,7 +6355,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>8</v>
       </c>
@@ -6406,7 +6417,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>8</v>
       </c>
@@ -6468,7 +6479,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>8</v>
       </c>
@@ -6530,7 +6541,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>9</v>
       </c>
@@ -6592,7 +6603,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>9</v>
       </c>
@@ -6654,7 +6665,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>9</v>
       </c>
@@ -6716,7 +6727,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>9</v>
       </c>
@@ -6778,7 +6789,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>9</v>
       </c>
@@ -6840,7 +6851,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>9</v>
       </c>
@@ -6902,7 +6913,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>9</v>
       </c>
@@ -6964,7 +6975,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>9</v>
       </c>
@@ -7026,7 +7037,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>9</v>
       </c>
@@ -7088,7 +7099,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>9</v>
       </c>
@@ -7150,7 +7161,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>9</v>
       </c>
@@ -7212,7 +7223,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>9</v>
       </c>
@@ -7274,7 +7285,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>9</v>
       </c>
@@ -7336,7 +7347,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>9</v>
       </c>
@@ -7398,7 +7409,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>9</v>
       </c>
@@ -7460,7 +7471,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>9</v>
       </c>
@@ -7522,7 +7533,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>9</v>
       </c>
@@ -7584,7 +7595,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>9</v>
       </c>
@@ -7646,7 +7657,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>9</v>
       </c>
@@ -7708,7 +7719,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>9</v>
       </c>
@@ -7770,7 +7781,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>9</v>
       </c>
@@ -7832,7 +7843,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>9</v>
       </c>
@@ -7894,7 +7905,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.15">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>9</v>
       </c>
@@ -7967,23 +7978,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3ED9FF6-8968-4FA6-BAEC-B95365AA2886}">
   <dimension ref="A1:O55"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.25" customWidth="1"/>
+    <col min="1" max="1" width="8.19921875" customWidth="1"/>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.69921875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="13.875" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="23.125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.8984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="23.09765625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="11.59765625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.75" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.25" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.25" customWidth="1"/>
+    <col min="12" max="12" width="9.69921875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.19921875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:15" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>180</v>
       </c>
@@ -7999,29 +8010,29 @@
       <c r="E1" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="4" t="str">
-        <f>LEFT(E1,LEN(E1)-5)&amp;VLOOKUP(LEFT(E1,LEN(E1)-5),Overzicht_variabelen!$A$2:$F$55,6,(FALSE))</f>
+      <c r="F1" s="6" t="str">
+        <f>LEFT(E1,LEN(E1)-5)&amp;VLOOKUP(LEFT(E1,LEN(E1)-5),Overzicht_variabelen!$A$2:$F$69,6,(FALSE))</f>
         <v>top_zand</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="4" t="str">
-        <f>LEFT(G1,LEN(G1)-5)&amp;VLOOKUP(LEFT(G1,LEN(G1)-5),Overzicht_variabelen!$A$2:$F$55,6,(FALSE))</f>
+      <c r="H1" s="6" t="str">
+        <f>LEFT(G1,LEN(G1)-5)&amp;VLOOKUP(LEFT(G1,LEN(G1)-5),Overzicht_variabelen!$A$2:$F$69,6,(FALSE))</f>
         <v>gamma_sat_deklaag_stdev</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="4" t="str">
-        <f>LEFT(I1,LEN(I1)-5)&amp;VLOOKUP(LEFT(I1,LEN(I1)-5),Overzicht_variabelen!$A$2:$F$55,6,(FALSE))</f>
+      <c r="J1" s="6" t="str">
+        <f>LEFT(I1,LEN(I1)-5)&amp;VLOOKUP(LEFT(I1,LEN(I1)-5),Overzicht_variabelen!$A$2:$F$69,6,(FALSE))</f>
         <v>D_wvp_stdev</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="L1" s="4" t="str">
-        <f>LEFT(K1,LEN(K1)-5)&amp;VLOOKUP(LEFT(K1,LEN(K1)-5),Overzicht_variabelen!$A$2:$F$55,6,(FALSE))</f>
+      <c r="L1" s="6" t="str">
+        <f>LEFT(K1,LEN(K1)-5)&amp;VLOOKUP(LEFT(K1,LEN(K1)-5),Overzicht_variabelen!$A$2:$F$69,6,(FALSE))</f>
         <v>kD_wvp_vc</v>
       </c>
       <c r="M1" s="4" t="s">
@@ -8030,12 +8041,12 @@
       <c r="N1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="O1" s="4" t="str">
-        <f>LEFT(N1,LEN(N1)-5)&amp;VLOOKUP(LEFT(N1,LEN(N1)-5),Overzicht_variabelen!$A$2:$F$55,6,(FALSE))</f>
+      <c r="O1" s="6" t="str">
+        <f>LEFT(N1,LEN(N1)-5)&amp;VLOOKUP(LEFT(N1,LEN(N1)-5),Overzicht_variabelen!$A$2:$F$69,6,(FALSE))</f>
         <v>d70_vc</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -8082,7 +8093,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -8129,7 +8140,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -8167,7 +8178,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
@@ -8200,7 +8211,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1</v>
       </c>
@@ -8233,7 +8244,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1</v>
       </c>
@@ -8266,7 +8277,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>2</v>
       </c>
@@ -8313,7 +8324,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2</v>
       </c>
@@ -8360,7 +8371,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2</v>
       </c>
@@ -8398,7 +8409,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2</v>
       </c>
@@ -8431,7 +8442,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2</v>
       </c>
@@ -8464,7 +8475,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2</v>
       </c>
@@ -8497,7 +8508,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>3</v>
       </c>
@@ -8544,7 +8555,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>3</v>
       </c>
@@ -8591,7 +8602,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>3</v>
       </c>
@@ -8629,7 +8640,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>3</v>
       </c>
@@ -8662,7 +8673,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>3</v>
       </c>
@@ -8695,7 +8706,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>3</v>
       </c>
@@ -8728,7 +8739,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>4</v>
       </c>
@@ -8775,7 +8786,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>4</v>
       </c>
@@ -8822,7 +8833,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>4</v>
       </c>
@@ -8860,7 +8871,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>4</v>
       </c>
@@ -8893,7 +8904,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>4</v>
       </c>
@@ -8926,7 +8937,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>4</v>
       </c>
@@ -8959,7 +8970,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>5</v>
       </c>
@@ -9006,7 +9017,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>5</v>
       </c>
@@ -9053,7 +9064,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>5</v>
       </c>
@@ -9091,7 +9102,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>5</v>
       </c>
@@ -9124,7 +9135,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>5</v>
       </c>
@@ -9157,7 +9168,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>5</v>
       </c>
@@ -9190,7 +9201,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>6</v>
       </c>
@@ -9237,7 +9248,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>6</v>
       </c>
@@ -9284,7 +9295,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>6</v>
       </c>
@@ -9322,7 +9333,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>6</v>
       </c>
@@ -9355,7 +9366,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>6</v>
       </c>
@@ -9388,7 +9399,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>6</v>
       </c>
@@ -9421,7 +9432,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>7</v>
       </c>
@@ -9468,7 +9479,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>7</v>
       </c>
@@ -9515,7 +9526,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>7</v>
       </c>
@@ -9553,7 +9564,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>7</v>
       </c>
@@ -9586,7 +9597,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>7</v>
       </c>
@@ -9619,7 +9630,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>7</v>
       </c>
@@ -9652,7 +9663,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>8</v>
       </c>
@@ -9699,7 +9710,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>8</v>
       </c>
@@ -9746,7 +9757,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>8</v>
       </c>
@@ -9784,7 +9795,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>8</v>
       </c>
@@ -9817,7 +9828,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>8</v>
       </c>
@@ -9850,7 +9861,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>8</v>
       </c>
@@ -9883,7 +9894,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>9</v>
       </c>
@@ -9930,7 +9941,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>9</v>
       </c>
@@ -9977,7 +9988,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>9</v>
       </c>
@@ -10015,7 +10026,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>9</v>
       </c>
@@ -10048,7 +10059,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>9</v>
       </c>
@@ -10081,7 +10092,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>9</v>
       </c>
@@ -10115,36 +10126,38 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:O1" xr:uid="{A3ED9FF6-8968-4FA6-BAEC-B95365AA2886}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9B7A8CE-63DA-4EEA-9A88-5E62FD2B5E40}">
-  <dimension ref="A1:R55"/>
-  <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.15"/>
+  <dimension ref="A1:R69"/>
+  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="71.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="71.09765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.19921875" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="23" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.375" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="17.19921875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.25" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.25" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.19921875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.19921875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="47.625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.25" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="47.59765625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.19921875" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>192</v>
       </c>
@@ -10197,7 +10210,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -10234,7 +10247,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>99</v>
       </c>
@@ -10262,7 +10275,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -10293,7 +10306,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>88</v>
       </c>
@@ -10313,7 +10326,7 @@
         <v>57</v>
       </c>
       <c r="I5" s="2">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="J5" s="2">
         <v>60</v>
@@ -10325,7 +10338,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>93</v>
       </c>
@@ -10348,7 +10361,7 @@
         <v>1.4999999999999999E-4</v>
       </c>
       <c r="J6" s="1">
-        <v>5.0000000000000001E-4</v>
+        <v>5</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>70</v>
@@ -10360,7 +10373,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>71</v>
       </c>
@@ -10380,7 +10393,7 @@
         <v>57</v>
       </c>
       <c r="I7" s="2">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J7" s="2">
         <v>22</v>
@@ -10389,7 +10402,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>84</v>
       </c>
@@ -10409,7 +10422,7 @@
         <v>59</v>
       </c>
       <c r="I8" s="2">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="J8" s="2">
         <v>4000</v>
@@ -10430,7 +10443,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -10465,7 +10478,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -10498,7 +10511,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -10534,7 +10547,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -10572,7 +10585,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>105</v>
       </c>
@@ -10606,7 +10619,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>106</v>
       </c>
@@ -10640,7 +10653,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>102</v>
       </c>
@@ -10674,7 +10687,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -10696,8 +10709,8 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.15">
-      <c r="A17" t="s">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A17" s="7" t="s">
         <v>19</v>
       </c>
       <c r="B17" t="s">
@@ -10709,15 +10722,11 @@
       <c r="D17" t="s">
         <v>53</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="I17" s="2">
-        <v>-4</v>
-      </c>
-      <c r="J17" s="2">
-        <v>15</v>
-      </c>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
       <c r="K17" s="2" t="s">
         <v>55</v>
       </c>
@@ -10725,7 +10734,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -10759,8 +10768,8 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.15">
-      <c r="A19" t="s">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A19" s="7" t="s">
         <v>67</v>
       </c>
       <c r="B19" t="s">
@@ -10772,7 +10781,7 @@
       <c r="D19" t="s">
         <v>53</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="7" t="s">
         <v>69</v>
       </c>
       <c r="I19" s="2">
@@ -10788,7 +10797,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>130</v>
       </c>
@@ -10817,7 +10826,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>115</v>
       </c>
@@ -10842,7 +10851,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>132</v>
       </c>
@@ -10870,7 +10879,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>138</v>
       </c>
@@ -10899,7 +10908,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>81</v>
       </c>
@@ -10922,7 +10931,7 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>178</v>
       </c>
@@ -10942,7 +10951,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>108</v>
       </c>
@@ -10976,7 +10985,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>174</v>
       </c>
@@ -10996,7 +11005,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>176</v>
       </c>
@@ -11016,7 +11025,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>111</v>
       </c>
@@ -11045,7 +11054,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>127</v>
       </c>
@@ -11074,7 +11083,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>135</v>
       </c>
@@ -11103,7 +11112,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>75</v>
       </c>
@@ -11125,7 +11134,7 @@
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>79</v>
       </c>
@@ -11149,7 +11158,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>146</v>
       </c>
@@ -11169,7 +11178,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>142</v>
       </c>
@@ -11189,7 +11198,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>140</v>
       </c>
@@ -11209,7 +11218,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>170</v>
       </c>
@@ -11229,7 +11238,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>172</v>
       </c>
@@ -11249,7 +11258,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>168</v>
       </c>
@@ -11269,7 +11278,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>122</v>
       </c>
@@ -11289,7 +11298,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>144</v>
       </c>
@@ -11309,7 +11318,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>90</v>
       </c>
@@ -11330,7 +11339,7 @@
       </c>
       <c r="K42" s="2"/>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>158</v>
       </c>
@@ -11350,7 +11359,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>125</v>
       </c>
@@ -11370,7 +11379,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>156</v>
       </c>
@@ -11390,7 +11399,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>162</v>
       </c>
@@ -11410,7 +11419,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>160</v>
       </c>
@@ -11430,7 +11439,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>120</v>
       </c>
@@ -11456,7 +11465,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>117</v>
       </c>
@@ -11476,7 +11485,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>166</v>
       </c>
@@ -11496,7 +11505,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>164</v>
       </c>
@@ -11516,7 +11525,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>154</v>
       </c>
@@ -11542,7 +11551,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>150</v>
       </c>
@@ -11562,7 +11571,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>152</v>
       </c>
@@ -11582,7 +11591,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>148</v>
       </c>
@@ -11602,9 +11611,93 @@
         <v>119</v>
       </c>
     </row>
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A56" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="K56" s="2"/>
+    </row>
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A57" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="K57" s="2"/>
+    </row>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A58" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="K58" s="2"/>
+    </row>
+    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A59" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K59" s="2"/>
+    </row>
+    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A60" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="K60" s="2"/>
+    </row>
+    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A61" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="K61" s="2"/>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A62" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="K62" s="2"/>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A63" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="K63" s="2"/>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A64" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="K64" s="2"/>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A65" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="K65" s="2"/>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A66" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="K66" s="2"/>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A67" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="K67" s="2"/>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A68" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="K68" s="2"/>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>185</v>
+      </c>
+      <c r="K69" s="2"/>
+    </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2 F3:F55" xr:uid="{0C4D3287-2227-4749-A999-A3EC2866277F}">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F55" xr:uid="{0C4D3287-2227-4749-A999-A3EC2866277F}">
       <formula1>$R$1:$R$2</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fixed adding variables to ReliabilityProject + improved input data checks
</commit_message>
<xml_diff>
--- a/workspaces/example_new_calculations/input/input.xlsx
+++ b/workspaces/example_new_calculations/input/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MKL\Documents\Github\GeoProb-Pipe\workspaces\example_new_calculations\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A649AE8-E2B8-467A-841A-3324CE662DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A6A4E11-75C2-4C05-96AC-7A229ADBDE58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-165" windowWidth="25440" windowHeight="15270" activeTab="3" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="233">
   <si>
     <t>M_van</t>
   </si>
@@ -676,9 +676,6 @@
   </si>
   <si>
     <t>variation_coefficient</t>
-  </si>
-  <si>
-    <t>start_value</t>
   </si>
   <si>
     <t>relaxation_factor</t>
@@ -8352,37 +8349,37 @@
   <sheetData>
     <row r="1" spans="1:16" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>231</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>232</v>
       </c>
       <c r="L1" s="4" t="s">
         <v>170</v>
@@ -8411,7 +8408,7 @@
         <v>189</v>
       </c>
       <c r="D2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
@@ -8428,7 +8425,7 @@
         <v>188</v>
       </c>
       <c r="D3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
@@ -8443,7 +8440,7 @@
         <v>190</v>
       </c>
       <c r="D4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
@@ -8458,7 +8455,7 @@
         <v>190</v>
       </c>
       <c r="D5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -8475,7 +8472,7 @@
         <v>190</v>
       </c>
       <c r="D6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -8492,7 +8489,7 @@
         <v>189</v>
       </c>
       <c r="D7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -8509,7 +8506,7 @@
         <v>186</v>
       </c>
       <c r="D8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -8526,7 +8523,7 @@
         <v>187</v>
       </c>
       <c r="D9" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -8543,7 +8540,7 @@
         <v>188</v>
       </c>
       <c r="D10" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -8558,7 +8555,7 @@
         <v>190</v>
       </c>
       <c r="D11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -8573,7 +8570,7 @@
         <v>190</v>
       </c>
       <c r="D12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -8590,7 +8587,7 @@
         <v>189</v>
       </c>
       <c r="D13" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
@@ -8607,7 +8604,7 @@
         <v>188</v>
       </c>
       <c r="D14" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -8624,7 +8621,7 @@
         <v>191</v>
       </c>
       <c r="D15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E15" t="s">
         <v>203</v>
@@ -8648,7 +8645,7 @@
         <v>52</v>
       </c>
       <c r="D16" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E16" t="s">
         <v>203</v>
@@ -8685,7 +8682,7 @@
         <v>79</v>
       </c>
       <c r="D17" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E17" t="s">
         <v>205</v>
@@ -8713,7 +8710,7 @@
         <v>79</v>
       </c>
       <c r="D18" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E18" t="s">
         <v>205</v>
@@ -8744,7 +8741,7 @@
         <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E19" t="s">
         <v>205</v>
@@ -8776,7 +8773,7 @@
         <v>47</v>
       </c>
       <c r="D20" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E20" t="s">
         <v>205</v>
@@ -8811,7 +8808,7 @@
         <v>59</v>
       </c>
       <c r="D21" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E21" t="s">
         <v>205</v>
@@ -8840,7 +8837,7 @@
         <v>68</v>
       </c>
       <c r="D22" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E22" t="s">
         <v>205</v>
@@ -8881,7 +8878,7 @@
         <v>47</v>
       </c>
       <c r="D23" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E23" t="s">
         <v>203</v>
@@ -8916,7 +8913,7 @@
         <v>47</v>
       </c>
       <c r="D24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E24" t="s">
         <v>203</v>
@@ -8949,7 +8946,7 @@
         <v>47</v>
       </c>
       <c r="D25" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E25" t="s">
         <v>203</v>
@@ -8985,7 +8982,7 @@
         <v>47</v>
       </c>
       <c r="D26" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E26" t="s">
         <v>203</v>
@@ -9023,7 +9020,7 @@
         <v>52</v>
       </c>
       <c r="D27" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E27" t="s">
         <v>203</v>
@@ -9045,7 +9042,7 @@
         <v>52</v>
       </c>
       <c r="D28" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E28" t="s">
         <v>203</v>
@@ -9074,7 +9071,7 @@
         <v>52</v>
       </c>
       <c r="D29" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E29" t="s">
         <v>203</v>
@@ -9108,7 +9105,7 @@
         <v>52</v>
       </c>
       <c r="D30" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E30" t="s">
         <v>56</v>
@@ -9140,7 +9137,7 @@
         <v>47</v>
       </c>
       <c r="D31" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E31" t="s">
         <v>203</v>
@@ -9169,7 +9166,7 @@
         <v>84</v>
       </c>
       <c r="D32" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E32" t="s">
         <v>203</v>
@@ -9194,7 +9191,7 @@
         <v>112</v>
       </c>
       <c r="D33" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E33" t="s">
         <v>203</v>
@@ -9222,7 +9219,7 @@
         <v>59</v>
       </c>
       <c r="D34" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E34" t="s">
         <v>203</v>
@@ -9251,7 +9248,7 @@
         <v>59</v>
       </c>
       <c r="D35" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E35" t="s">
         <v>203</v>
@@ -9276,7 +9273,7 @@
         <v>47</v>
       </c>
       <c r="D36" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E36" t="s">
         <v>203</v>
@@ -9299,7 +9296,7 @@
         <v>84</v>
       </c>
       <c r="D37" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E37" t="s">
         <v>205</v>
@@ -9333,7 +9330,7 @@
         <v>73</v>
       </c>
       <c r="D38" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E38" t="s">
         <v>205</v>
@@ -9359,7 +9356,7 @@
         <v>73</v>
       </c>
       <c r="D39" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E39" t="s">
         <v>205</v>
@@ -9385,7 +9382,7 @@
         <v>84</v>
       </c>
       <c r="D40" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E40" t="s">
         <v>203</v>
@@ -9414,7 +9411,7 @@
         <v>107</v>
       </c>
       <c r="D41" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E41" t="s">
         <v>203</v>
@@ -9443,7 +9440,7 @@
         <v>115</v>
       </c>
       <c r="D42" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E42" t="s">
         <v>203</v>
@@ -9472,7 +9469,7 @@
         <v>84</v>
       </c>
       <c r="D43" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E43" t="s">
         <v>205</v>
@@ -9506,7 +9503,7 @@
         <v>84</v>
       </c>
       <c r="D44" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E44" t="s">
         <v>205</v>
@@ -9540,7 +9537,7 @@
         <v>84</v>
       </c>
       <c r="D45" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E45" t="s">
         <v>205</v>
@@ -10142,7 +10139,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F7FD5E8-359B-4F56-B38E-FCA72B85D698}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.09765625" style="7" bestFit="1" customWidth="1"/>
@@ -10151,29 +10148,29 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B3" s="7">
         <v>0.75</v>
@@ -10184,10 +10181,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B4" s="7">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>210</v>
@@ -10195,50 +10192,39 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B5" s="7">
-        <v>0.01</v>
+        <v>100</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="B6" s="7">
-        <v>100</v>
+        <v>207</v>
+      </c>
+      <c r="B6" s="7" t="b">
+        <v>1</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="B7" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" s="7" t="s">
         <v>206</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6" xr:uid="{94AA1909-8159-4ABD-8194-E5CC31B00066}">
-      <formula1>AND(ISNUMBER(B6),B6=INT(B6))</formula1>
-    </dataValidation>
-    <dataValidation type="custom" showInputMessage="1" showErrorMessage="1" sqref="B3:B5" xr:uid="{0F940659-071E-4396-94AE-334C05124B18}">
-      <formula1>ISNUMBER(B3)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5" xr:uid="{94AA1909-8159-4ABD-8194-E5CC31B00066}">
+      <formula1>AND(ISNUMBER(B5),B5=INT(B5))</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{73A82C8D-457E-4F26-8920-E365EC9333FD}">
       <formula1>"form,numerical_integration,crude_monte_carlo,importance_sampling,directional_sampling,subset_simulation,numerical_bisection,latin_hypercube,cobyla_reliability,form_then_directional_sampling,directional_sampling_then_form"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7" xr:uid="{05F071D7-CE12-4A8B-B2AB-37DFC65D1C77}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6" xr:uid="{05F071D7-CE12-4A8B-B2AB-37DFC65D1C77}">
       <formula1>"True,False"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" showInputMessage="1" showErrorMessage="1" sqref="B3:B4" xr:uid="{0F940659-071E-4396-94AE-334C05124B18}">
+      <formula1>ISNUMBER(B3)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
nog niet volledig werkend
</commit_message>
<xml_diff>
--- a/workspaces/example_new_calculations/input/input.xlsx
+++ b/workspaces/example_new_calculations/input/input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oscop\Documents\GeoProb-Pipe\workspaces\example_new_calculations\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\workspaces\example_new_calculations\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FB427C6-6B29-41A0-A209-FAFB22771210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BFE16AE-3D80-4E4F-8280-91C0922CECC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
   </bookViews>
   <sheets>
     <sheet name="Vakken" sheetId="1" r:id="rId1"/>
@@ -9271,6 +9271,9 @@
       <c r="G37">
         <v>0.1</v>
       </c>
+      <c r="H37">
+        <v>0.1</v>
+      </c>
       <c r="K37" s="2" t="s">
         <v>75</v>
       </c>
@@ -9296,6 +9299,9 @@
       </c>
       <c r="G38">
         <v>0.01</v>
+      </c>
+      <c r="H38">
+        <v>0.1</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>75</v>

</xml_diff>

<commit_message>
Naar single project (#10)
* Single project system builder implemented, now ready for testing

* nog niet volledig werkend

* Small change in collect_todos-script

* Small change in collect_todos-script

* Small change in collect_todos-script

* Small change in collect_todos-script

* Exporteren resultaten klaar, structuur verbetered. Verder opruimen nog wel nodig

* Voorlopig afgerond

* fixed some small mistakes
</commit_message>
<xml_diff>
--- a/workspaces/example_new_calculations/input/input.xlsx
+++ b/workspaces/example_new_calculations/input/input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oscop\Documents\GeoProb-Pipe\workspaces\example_new_calculations\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\workspaces\example_new_calculations\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FB427C6-6B29-41A0-A209-FAFB22771210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BFE16AE-3D80-4E4F-8280-91C0922CECC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{E14FA4F5-43AA-4DAE-BCE2-7688F4F5853B}"/>
   </bookViews>
   <sheets>
     <sheet name="Vakken" sheetId="1" r:id="rId1"/>
@@ -9271,6 +9271,9 @@
       <c r="G37">
         <v>0.1</v>
       </c>
+      <c r="H37">
+        <v>0.1</v>
+      </c>
       <c r="K37" s="2" t="s">
         <v>75</v>
       </c>
@@ -9296,6 +9299,9 @@
       </c>
       <c r="G38">
         <v>0.01</v>
+      </c>
+      <c r="H38">
+        <v>0.1</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>75</v>

</xml_diff>